<commit_message>
Plots raw and updates to markdown GF
</commit_message>
<xml_diff>
--- a/CPRD Raw Analysis/Results/AttritionReportCoh_Raw.xlsx
+++ b/CPRD Raw Analysis/Results/AttritionReportCoh_Raw.xlsx
@@ -351,313 +351,486 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E16"/>
+  <dimension ref="A1:F16"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>number_records</t>
+          <t>Reason for exclusion</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>number_subjects</t>
+          <t>Number of records</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>reason</t>
+          <t>Number of subjects</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>subjects_excluded</t>
+          <t>N subjects excluded</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>records_excluded</t>
+          <t>Perc subjects excluded (%)</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>N records excluded</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2">
-        <v>57617</v>
-      </c>
-      <c r="B2">
-        <v>31217</v>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Had their 1st fx &gt;= 01/04/2012 and &lt;= 31/03/2018 when they were &gt; 50 years old</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>57,617</t>
+        </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Had their 1st fx &gt;= 01/04/2012 and &lt;= 31/03/2018 when they were &gt; 50 years old</t>
+          <t>31,217</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>NA</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3">
-        <v>57617</v>
-      </c>
-      <c r="B3">
-        <v>31217</v>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Excluding fracture happening before the birth year</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>57,617</t>
+        </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Excluding fracture happening before the birth year</t>
-        </is>
-      </c>
-      <c r="D3">
-        <v>0</v>
+          <t>31,217</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="E3">
         <v>0</v>
       </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
     </row>
     <row r="4">
-      <c r="A4">
-        <v>53050</v>
-      </c>
-      <c r="B4">
-        <v>31217</v>
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Excluding records that happen outside of study period</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>53,050</t>
+        </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Excluding records that happen outside of study period</t>
-        </is>
-      </c>
-      <c r="D4">
+          <t>31,217</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E4">
         <v>0</v>
       </c>
-      <c r="E4">
-        <v>4567</v>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>4,567</t>
+        </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5">
-        <v>53003</v>
-      </c>
-      <c r="B5">
-        <v>31192</v>
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Excluding records that happen outside of observation period</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>53,003</t>
+        </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Excluding records that happen outside of observation period</t>
-        </is>
-      </c>
-      <c r="D5">
-        <v>25</v>
+          <t>31,192</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
       </c>
       <c r="E5">
-        <v>47</v>
+        <v>0.08</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>47</t>
+        </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6">
-        <v>47097</v>
-      </c>
-      <c r="B6">
-        <v>30543</v>
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Excluding trauma fractures (same day as trauma codes or 3 distinct fracture sites on the same date</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>47,097</t>
+        </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Excluding trauma fractures (same day as trauma codes or 3 distinct fracture sites on the same date</t>
-        </is>
-      </c>
-      <c r="D6">
-        <v>649</v>
+          <t>30,543</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>649</t>
+        </is>
       </c>
       <c r="E6">
-        <v>5906</v>
+        <v>2.08</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>5,906</t>
+        </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7">
-        <v>47086</v>
-      </c>
-      <c r="B7">
-        <v>30536</v>
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Excluding fractures on the same day as death or after death</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>47,086</t>
+        </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Excluding fractures on the same day as death or after death</t>
-        </is>
-      </c>
-      <c r="D7">
-        <v>7</v>
+          <t>30,536</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
       </c>
       <c r="E7">
-        <v>11</v>
+        <v>0.02</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8">
-        <v>35926</v>
-      </c>
-      <c r="B8">
-        <v>30536</v>
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Clean out using washout period</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>35,926</t>
+        </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Clean out using washout period</t>
-        </is>
-      </c>
-      <c r="D8">
+          <t>30,536</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E8">
         <v>0</v>
       </c>
-      <c r="E8">
-        <v>11160</v>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>11,160</t>
+        </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9">
-        <v>33957</v>
-      </c>
-      <c r="B9">
-        <v>30536</v>
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Excluding records on the same day for the same person according to hierarchy (Hip, Spine, NHNS)</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>33,957</t>
+        </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Excluding records on the same day for the same person according to hierarchy (Hip, Spine, NHNS)</t>
-        </is>
-      </c>
-      <c r="D9">
+          <t>30,536</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E9">
         <v>0</v>
       </c>
-      <c r="E9">
-        <v>1969</v>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>1,969</t>
+        </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10">
-        <v>33957</v>
-      </c>
-      <c r="B10">
-        <v>30536</v>
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Excluding not female individuals</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>33,957</t>
+        </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Excluding not female individuals</t>
-        </is>
-      </c>
-      <c r="D10">
-        <v>0</v>
+          <t>30,536</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="E10">
         <v>0</v>
       </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
     </row>
     <row r="11">
-      <c r="A11">
-        <v>33957</v>
-      </c>
-      <c r="B11">
-        <v>30536</v>
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Excluding individuals without fracture records</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>33,957</t>
+        </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Excluding individuals without fracture records</t>
-        </is>
-      </c>
-      <c r="D11">
-        <v>0</v>
+          <t>30,536</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="E11">
         <v>0</v>
       </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
     </row>
     <row r="12">
-      <c r="A12">
-        <v>30528</v>
-      </c>
-      <c r="B12">
-        <v>30528</v>
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Excluding index fractures that happen on the last day of observation period</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>30,528</t>
+        </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Excluding index fractures that happen on the last day of observation period</t>
-        </is>
-      </c>
-      <c r="D12">
-        <v>8</v>
+          <t>30,528</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
       </c>
       <c r="E12">
-        <v>3429</v>
+        <v>0.03</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>3,429</t>
+        </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13">
-        <v>27078</v>
-      </c>
-      <c r="B13">
-        <v>27078</v>
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Excluding records with insufficient prior observation and/or outside of observation period</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>27,078</t>
+        </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Excluding records with insufficient prior observation and/or outside of observation period</t>
-        </is>
-      </c>
-      <c r="D13">
-        <v>3450</v>
+          <t>27,078</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>3,450</t>
+        </is>
       </c>
       <c r="E13">
-        <v>3450</v>
+        <v>11.3</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>3,450</t>
+        </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14">
-        <v>27078</v>
-      </c>
-      <c r="B14">
-        <v>27078</v>
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Excluding records of index fractures where the subject has not turned 50</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>27,078</t>
+        </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Excluding records of index fractures where the subject has not turned 50</t>
-        </is>
-      </c>
-      <c r="D14">
-        <v>0</v>
+          <t>27,078</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="E14">
         <v>0</v>
       </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
     </row>
     <row r="15">
-      <c r="A15">
-        <v>25264</v>
-      </c>
-      <c r="B15">
-        <v>25264</v>
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Excluding records happened after cancer</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>25,264</t>
+        </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Excluding records happened after cancer</t>
-        </is>
-      </c>
-      <c r="D15">
-        <v>1814</v>
+          <t>25,264</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>1,814</t>
+        </is>
       </c>
       <c r="E15">
-        <v>1814</v>
+        <v>6.7</v>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>1,814</t>
+        </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16">
-        <v>25138</v>
-      </c>
-      <c r="B16">
-        <v>25138</v>
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Excluding records happened after metabolic bone diseases</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>25,138</t>
+        </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Excluding records happened after metabolic bone diseases</t>
-        </is>
-      </c>
-      <c r="D16">
-        <v>126</v>
+          <t>25,138</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>126</t>
+        </is>
       </c>
       <c r="E16">
-        <v>126</v>
+        <v>0.5</v>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>126</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>